<commit_message>
Refine report design, budget comparisons and tooltips
</commit_message>
<xml_diff>
--- a/powerbi-ledningsrapport/data/Budgetscenarier.xlsx
+++ b/powerbi-ledningsrapport/data/Budgetscenarier.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="125" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,20 @@
       <c r="A12" t="inlineStr">
         <is>
           <t>Ändra sökvägen via Power Query-parametern BudgetWorkbook. Utfall ändras aldrig här.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Detaljvariation v1: huvudgruppernas månadsbudgetar är oförändrade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Underkategorier har olika konto- och månadsprofiler. Utfall och huvudgruppernas totaler har inte ändrats.</t>
         </is>
       </c>
     </row>
@@ -811,40 +825,40 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4322500</v>
+        <v>4134865</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>4227500</v>
+        <v>4350358</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>4892500</v>
+        <v>5024496</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>4940000</v>
+        <v>5321318</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>5130000</v>
+        <v>4901403</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>5177500</v>
+        <v>4963800</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>3847500</v>
+        <v>3953842</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>4892500</v>
+        <v>5018478</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>5367500</v>
+        <v>5121798</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>5177500</v>
+        <v>4958415</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>4892500</v>
+        <v>5031117</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>5130000</v>
+        <v>5265175</v>
       </c>
     </row>
     <row r="3">
@@ -863,40 +877,40 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1512875</v>
+        <v>1720998</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1479625</v>
+        <v>1294231</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1712375</v>
+        <v>1513191</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1729000</v>
+        <v>1619532</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1795500</v>
+        <v>2049058</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>1812125</v>
+        <v>2049159</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>1346625</v>
+        <v>1186153</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>1712375</v>
+        <v>1522272</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>1878625</v>
+        <v>2151155</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1812125</v>
+        <v>2055132</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>1712375</v>
+        <v>1503200</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>1795500</v>
+        <v>1591519</v>
       </c>
     </row>
     <row r="4">
@@ -915,40 +929,40 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1167075</v>
+        <v>1146587</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1141425</v>
+        <v>1203961</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1320975</v>
+        <v>1388163</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1333800</v>
+        <v>1061950</v>
       </c>
       <c r="I4" s="2" t="n">
+        <v>1360139</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>1374591</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>1092955</v>
+      </c>
+      <c r="L4" s="2" t="n">
         <v>1385100</v>
       </c>
-      <c r="J4" s="2" t="n">
-        <v>1397925</v>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>1038825</v>
-      </c>
-      <c r="L4" s="2" t="n">
-        <v>1320975</v>
-      </c>
       <c r="M4" s="2" t="n">
-        <v>1449225</v>
+        <v>1422397</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1397925</v>
+        <v>1374003</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>1320975</v>
+        <v>1391533</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1385100</v>
+        <v>1453906</v>
       </c>
     </row>
     <row r="5">
@@ -967,40 +981,40 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-2683176</v>
+        <v>-2808862</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-2624206</v>
+        <v>-2830469</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-3037002</v>
+        <v>-2826515</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>-3066487</v>
+        <v>-2915250</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-3184429</v>
+        <v>-3337317</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>-3213915</v>
+        <v>-3399373</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>-2388322</v>
+        <v>-2218400</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>-3037002</v>
+        <v>-2836863</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-3331856</v>
+        <v>-3495917</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-3213915</v>
+        <v>-3360884</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>-3037002</v>
+        <v>-2815038</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>-3184429</v>
+        <v>-2969286</v>
       </c>
     </row>
     <row r="6">
@@ -1019,40 +1033,40 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-1520226</v>
+        <v>-1369376</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-1486814</v>
+        <v>-1394503</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-1720695</v>
+        <v>-1912828</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>-1737400</v>
+        <v>-1948174</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>-1804224</v>
+        <v>-1620726</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>-1820929</v>
+        <v>-1669204</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>-1353169</v>
+        <v>-1508274</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>-1720695</v>
+        <v>-1903383</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>-1887753</v>
+        <v>-1690846</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-1820929</v>
+        <v>-1644535</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>-1720695</v>
+        <v>-1923304</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>-1804224</v>
+        <v>-2000607</v>
       </c>
     </row>
     <row r="7">
@@ -1071,40 +1085,40 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-345496</v>
+        <v>-370091</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-337904</v>
+        <v>-269386</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>-391056</v>
+        <v>-374063</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>-394853</v>
+        <v>-385004</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>-410039</v>
+        <v>-439957</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>-413837</v>
+        <v>-447444</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>-307529</v>
+        <v>-293811</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>-391056</v>
+        <v>-374898</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-429023</v>
+        <v>-461127</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-413837</v>
+        <v>-442597</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>-391056</v>
+        <v>-373136</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>-410039</v>
+        <v>-392670</v>
       </c>
     </row>
     <row r="8">
@@ -1123,40 +1137,40 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-253275</v>
+        <v>-234309</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-247708</v>
+        <v>-238137</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>-286674</v>
+        <v>-326095</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>-289458</v>
+        <v>-239902</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-300590</v>
+        <v>-277519</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-303373</v>
+        <v>-285226</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>-225442</v>
+        <v>-257266</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>-286674</v>
+        <v>-324157</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>-314506</v>
+        <v>-289749</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-303373</v>
+        <v>-281195</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>-286674</v>
+        <v>-328245</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>-300590</v>
+        <v>-340883</v>
       </c>
     </row>
     <row r="9">
@@ -1175,40 +1189,40 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-204483</v>
+        <v>-224018</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-199989</v>
+        <v>-164126</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-231448</v>
+        <v>-227374</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-233695</v>
+        <v>-233563</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>-242684</v>
+        <v>-266447</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>-244930</v>
+        <v>-195737</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>-182012</v>
+        <v>-178723</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>-231448</v>
+        <v>-227574</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>-253918</v>
+        <v>-279417</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-244930</v>
+        <v>-267773</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>-231448</v>
+        <v>-227152</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>-242684</v>
+        <v>-238520</v>
       </c>
     </row>
     <row r="10">
@@ -1279,40 +1293,40 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-317616</v>
+        <v>-329398</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-310635</v>
+        <v>-332636</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-359499</v>
+        <v>-328625</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-362988</v>
+        <v>-352983</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-376950</v>
+        <v>-391289</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-380440</v>
+        <v>-393889</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>-282713</v>
+        <v>-257783</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-359499</v>
+        <v>-330158</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-394401</v>
+        <v>-409793</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-380440</v>
+        <v>-394214</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>-359499</v>
+        <v>-394507</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>-376950</v>
+        <v>-345402</v>
       </c>
     </row>
     <row r="12">
@@ -1331,40 +1345,40 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-103947</v>
+        <v>-92403</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-101662</v>
+        <v>-94347</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-117654</v>
+        <v>-129060</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>-118796</v>
+        <v>-136802</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-123365</v>
+        <v>-109317</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>-124508</v>
+        <v>-111331</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>-92524</v>
+        <v>-101734</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>-117654</v>
+        <v>-128494</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>-129077</v>
+        <v>-113997</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-124508</v>
+        <v>-111013</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>-117654</v>
+        <v>-112270</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>-123365</v>
+        <v>-135020</v>
       </c>
     </row>
     <row r="13">
@@ -1383,40 +1397,40 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-62368</v>
+        <v>-66222</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-60997</v>
+        <v>-66769</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-70593</v>
+        <v>-66374</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>-71277</v>
+        <v>-71136</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>-74019</v>
+        <v>-78708</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>-74705</v>
+        <v>-79104</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>-55515</v>
+        <v>-52108</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>-70593</v>
+        <v>-66584</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-77446</v>
+        <v>-82480</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-74705</v>
+        <v>-79210</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>-70593</v>
+        <v>-57258</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>-74019</v>
+        <v>-69708</v>
       </c>
     </row>
     <row r="14">
@@ -1435,40 +1449,40 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-41579</v>
+        <v>-37988</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-40665</v>
+        <v>-38707</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-47062</v>
+        <v>-52854</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>-47519</v>
+        <v>-55937</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>-49346</v>
+        <v>-44976</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>-49803</v>
+        <v>-45704</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>-37010</v>
+        <v>-41687</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>-47062</v>
+        <v>-52566</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>-51631</v>
+        <v>-46940</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-49803</v>
+        <v>-45605</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>-47062</v>
+        <v>-46031</v>
       </c>
       <c r="P14" s="2" t="n">
-        <v>-49346</v>
+        <v>-55264</v>
       </c>
     </row>
     <row r="15">
@@ -1487,40 +1501,40 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-83158</v>
+        <v>-90350</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-81330</v>
+        <v>-65802</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>-94124</v>
+        <v>-90957</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>-95037</v>
+        <v>-97281</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>-98692</v>
+        <v>-107443</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>-99607</v>
+        <v>-107816</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>-74019</v>
+        <v>-71462</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>-94124</v>
+        <v>-91114</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>-103261</v>
+        <v>-112655</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-99607</v>
+        <v>-108014</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>-94124</v>
+        <v>-78590</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>-98692</v>
+        <v>-95456</v>
       </c>
     </row>
     <row r="16">
@@ -1539,40 +1553,40 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>-124735</v>
+        <v>-117042</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-121995</v>
+        <v>-119023</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>-141184</v>
+        <v>-162246</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>-142556</v>
+        <v>-124034</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>-148040</v>
+        <v>-138679</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>-149409</v>
+        <v>-140628</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>-111029</v>
+        <v>-128036</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>-141184</v>
+        <v>-161200</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>-154892</v>
+        <v>-144843</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-149409</v>
+        <v>-140416</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>-141184</v>
+        <v>-141460</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>-148040</v>
+        <v>-169562</v>
       </c>
     </row>
     <row r="17">
@@ -1760,40 +1774,40 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4603463</v>
+        <v>4403632</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>4502288</v>
+        <v>4633131</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>5210513</v>
+        <v>5351089</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>5261100</v>
+        <v>5667204</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>5463450</v>
+        <v>5219993</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>5514038</v>
+        <v>5286448</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>4097588</v>
+        <v>4210843</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>5210513</v>
+        <v>5344680</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>5716388</v>
+        <v>5454715</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>4363160</v>
+        <v>4193047</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>3926844</v>
+        <v>4019990</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>4363160</v>
+        <v>4459443</v>
       </c>
     </row>
     <row r="3">
@@ -1812,40 +1826,40 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1611211</v>
+        <v>1832862</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1575801</v>
+        <v>1378357</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1823679</v>
+        <v>1611548</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1841385</v>
+        <v>1724801</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1912208</v>
+        <v>2182248</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>1929914</v>
+        <v>2182355</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>1434156</v>
+        <v>1263253</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>1823679</v>
+        <v>1621219</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>2000735</v>
+        <v>2290980</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1374695</v>
+        <v>1564458</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>1237225</v>
+        <v>1081220</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>1374695</v>
+        <v>1213436</v>
       </c>
     </row>
     <row r="4">
@@ -1864,40 +1878,40 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1242934</v>
+        <v>1221114</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1215618</v>
+        <v>1282219</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1406838</v>
+        <v>1478393</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1420497</v>
+        <v>1130977</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1475132</v>
+        <v>1448549</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1488791</v>
+        <v>1463940</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1106349</v>
+        <v>1163997</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>1406838</v>
+        <v>1475131</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1543424</v>
+        <v>1514852</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1434463</v>
+        <v>1414813</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>1291017</v>
+        <v>1353876</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1434463</v>
+        <v>1499439</v>
       </c>
     </row>
     <row r="5">
@@ -1916,40 +1930,40 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-2857582</v>
+        <v>-2991437</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-2794779</v>
+        <v>-3014449</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-3234406</v>
+        <v>-3010237</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>-3265809</v>
+        <v>-3104741</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-3391417</v>
+        <v>-3554243</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>-3422819</v>
+        <v>-3620332</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>-2543563</v>
+        <v>-2362596</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>-3234406</v>
+        <v>-3021258</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-3548427</v>
+        <v>-3723152</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-2714392</v>
+        <v>-2843647</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>-2415553</v>
+        <v>-2233567</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>-2682361</v>
+        <v>-2494686</v>
       </c>
     </row>
     <row r="6">
@@ -1968,40 +1982,40 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-1619040</v>
+        <v>-1458385</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-1583456</v>
+        <v>-1485145</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-1832539</v>
+        <v>-2037161</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>-1850332</v>
+        <v>-2074806</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>-1921498</v>
+        <v>-1726073</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>-1939291</v>
+        <v>-1777704</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>-1441124</v>
+        <v>-1606311</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>-1832539</v>
+        <v>-2027101</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>-2010456</v>
+        <v>-1800750</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-1621119</v>
+        <v>-1466726</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>-1463647</v>
+        <v>-1632013</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>-1641366</v>
+        <v>-1815329</v>
       </c>
     </row>
     <row r="7">
@@ -2020,40 +2034,40 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-367953</v>
+        <v>-394147</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-359867</v>
+        <v>-286895</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>-416475</v>
+        <v>-398377</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>-420518</v>
+        <v>-410029</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>-436692</v>
+        <v>-468555</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>-440736</v>
+        <v>-476528</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>-327520</v>
+        <v>-312910</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>-416475</v>
+        <v>-399267</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-456909</v>
+        <v>-491100</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-332861</v>
+        <v>-356637</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>-298555</v>
+        <v>-284181</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>-333976</v>
+        <v>-319004</v>
       </c>
     </row>
     <row r="8">
@@ -2072,40 +2086,40 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-269738</v>
+        <v>-249539</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-263810</v>
+        <v>-253617</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>-305308</v>
+        <v>-347292</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>-308271</v>
+        <v>-255495</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-320129</v>
+        <v>-295558</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-323093</v>
+        <v>-303766</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>-240096</v>
+        <v>-273989</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>-305308</v>
+        <v>-345228</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>-334950</v>
+        <v>-308584</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-250078</v>
+        <v>-232215</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>-223649</v>
+        <v>-255458</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>-249430</v>
+        <v>-282136</v>
       </c>
     </row>
     <row r="9">
@@ -2124,40 +2138,40 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-217775</v>
+        <v>-238580</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-212989</v>
+        <v>-174795</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-246492</v>
+        <v>-242153</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-248886</v>
+        <v>-248745</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>-258458</v>
+        <v>-283765</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>-260850</v>
+        <v>-208459</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>-193844</v>
+        <v>-190341</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>-246492</v>
+        <v>-242366</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>-270423</v>
+        <v>-297579</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-201864</v>
+        <v>-221089</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>-182112</v>
+        <v>-178297</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>-204249</v>
+        <v>-200227</v>
       </c>
     </row>
     <row r="10">
@@ -2228,40 +2242,40 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-338260</v>
+        <v>-350809</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-330826</v>
+        <v>-354257</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-382866</v>
+        <v>-349986</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-386583</v>
+        <v>-375928</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-401452</v>
+        <v>-416723</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-405170</v>
+        <v>-419494</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>-301089</v>
+        <v>-274537</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-382866</v>
+        <v>-351618</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-420037</v>
+        <v>-436429</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-319949</v>
+        <v>-331533</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>-293402</v>
+        <v>-321973</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>-321914</v>
+        <v>-294972</v>
       </c>
     </row>
     <row r="12">
@@ -2280,40 +2294,40 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-110704</v>
+        <v>-98409</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-108271</v>
+        <v>-100481</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-125302</v>
+        <v>-137449</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>-126518</v>
+        <v>-145694</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-131384</v>
+        <v>-116423</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>-132601</v>
+        <v>-118567</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>-98538</v>
+        <v>-108347</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>-125302</v>
+        <v>-136846</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>-137467</v>
+        <v>-121407</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-104710</v>
+        <v>-93361</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>-96023</v>
+        <v>-91629</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>-105353</v>
+        <v>-115306</v>
       </c>
     </row>
     <row r="13">
@@ -2332,40 +2346,40 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-66422</v>
+        <v>-70526</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-64962</v>
+        <v>-71109</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-75181</v>
+        <v>-70688</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>-75911</v>
+        <v>-75761</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>-78830</v>
+        <v>-83824</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>-79561</v>
+        <v>-84246</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>-59123</v>
+        <v>-55495</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>-75181</v>
+        <v>-70911</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-82480</v>
+        <v>-87841</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-62826</v>
+        <v>-66614</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>-57613</v>
+        <v>-46730</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>-63212</v>
+        <v>-59530</v>
       </c>
     </row>
     <row r="14">
@@ -2384,40 +2398,40 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-44281</v>
+        <v>-40457</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-43308</v>
+        <v>-41223</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-50121</v>
+        <v>-56289</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>-50607</v>
+        <v>-59572</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>-52554</v>
+        <v>-47900</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>-53040</v>
+        <v>-48675</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>-39415</v>
+        <v>-44396</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>-50121</v>
+        <v>-55983</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>-54986</v>
+        <v>-49990</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-41884</v>
+        <v>-38354</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>-38409</v>
+        <v>-37568</v>
       </c>
       <c r="P14" s="2" t="n">
-        <v>-42141</v>
+        <v>-47195</v>
       </c>
     </row>
     <row r="15">
@@ -2436,40 +2450,40 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-88563</v>
+        <v>-96222</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-86616</v>
+        <v>-70078</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>-100241</v>
+        <v>-96868</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>-101215</v>
+        <v>-103605</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>-105107</v>
+        <v>-114427</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>-106081</v>
+        <v>-114823</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>-78830</v>
+        <v>-76107</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>-100241</v>
+        <v>-97036</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>-109973</v>
+        <v>-119978</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-83768</v>
+        <v>-90838</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>-76818</v>
+        <v>-64140</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>-84283</v>
+        <v>-81520</v>
       </c>
     </row>
     <row r="16">
@@ -2488,40 +2502,40 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>-132844</v>
+        <v>-124651</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-129924</v>
+        <v>-126759</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>-150361</v>
+        <v>-172792</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>-151822</v>
+        <v>-132096</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>-157661</v>
+        <v>-147691</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>-159121</v>
+        <v>-149769</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>-118245</v>
+        <v>-136358</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>-150361</v>
+        <v>-171678</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>-164961</v>
+        <v>-154259</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-125653</v>
+        <v>-118090</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>-115227</v>
+        <v>-115452</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>-126424</v>
+        <v>-144804</v>
       </c>
     </row>
     <row r="17">
@@ -2709,40 +2723,40 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4654037</v>
+        <v>4467876</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>4993394</v>
+        <v>5114872</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>5672108</v>
+        <v>5800253</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>5962985</v>
+        <v>6461656</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>6326581</v>
+        <v>6066777</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>6835617</v>
+        <v>6575681</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>6884096</v>
+        <v>7043411</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>7465851</v>
+        <v>7626862</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>7902167</v>
+        <v>7568780</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>5080392</v>
+        <v>4865172</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>4572352</v>
+        <v>4700138</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>5080391</v>
+        <v>5212443</v>
       </c>
     </row>
     <row r="3">
@@ -2761,40 +2775,40 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1466340</v>
+        <v>1674005</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1573261</v>
+        <v>1369805</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1787102</v>
+        <v>1572480</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1878749</v>
+        <v>1770317</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1993306</v>
+        <v>2283121</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2153687</v>
+        <v>2443649</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>2168962</v>
+        <v>1902135</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>2352255</v>
+        <v>2082587</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>2489724</v>
+        <v>2861621</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1793079</v>
+        <v>2033430</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>1613772</v>
+        <v>1416111</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>1793079</v>
+        <v>1588819</v>
       </c>
     </row>
     <row r="4">
@@ -2813,40 +2827,40 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1530095</v>
+        <v>1508591</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1641664</v>
+        <v>1723642</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1864803</v>
+        <v>1951280</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1960433</v>
+        <v>1570194</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>2079973</v>
+        <v>2049962</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2247327</v>
+        <v>2217301</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>2263265</v>
+        <v>2370777</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>2454526</v>
+        <v>2563183</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>2597973</v>
+        <v>2559463</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1464348</v>
+        <v>1439217</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>1317913</v>
+        <v>1387788</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1464348</v>
+        <v>1536556</v>
       </c>
     </row>
     <row r="5">
@@ -2865,40 +2879,40 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-2891828</v>
+        <v>-3034442</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-3140036</v>
+        <v>-3388283</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-3575330</v>
+        <v>-3322054</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>-3723733</v>
+        <v>-3532462</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-3901248</v>
+        <v>-4097423</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>-4197361</v>
+        <v>-4448751</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>-4261687</v>
+        <v>-3947925</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>-4681750</v>
+        <v>-4364157</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-4984222</v>
+        <v>-5239396</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-3172306</v>
+        <v>-3324277</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>-2823250</v>
+        <v>-2608304</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>-3135287</v>
+        <v>-2913861</v>
       </c>
     </row>
     <row r="6">
@@ -2917,40 +2931,40 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-1762686</v>
+        <v>-1591530</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-1887734</v>
+        <v>-1771283</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-2125554</v>
+        <v>-2359004</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>-2217390</v>
+        <v>-2481043</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>-2353849</v>
+        <v>-2119040</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>-2564379</v>
+        <v>-2355570</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>-2604210</v>
+        <v>-2894973</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>-2826559</v>
+        <v>-3120177</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>-2969506</v>
+        <v>-2664724</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-1945696</v>
+        <v>-1760873</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>-1752011</v>
+        <v>-1951869</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>-1959892</v>
+        <v>-2166081</v>
       </c>
     </row>
     <row r="7">
@@ -2969,40 +2983,40 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-360042</v>
+        <v>-386584</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-388127</v>
+        <v>-309556</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>-438500</v>
+        <v>-418754</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>-456093</v>
+        <v>-443760</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>-480949</v>
+        <v>-517161</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>-521808</v>
+        <v>-565351</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>-531077</v>
+        <v>-506033</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>-580119</v>
+        <v>-554997</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-612392</v>
+        <v>-659445</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-413343</v>
+        <v>-442989</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>-370525</v>
+        <v>-352383</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>-414357</v>
+        <v>-395501</v>
       </c>
     </row>
     <row r="8">
@@ -3021,40 +3035,40 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-268815</v>
+        <v>-249273</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-290546</v>
+        <v>-279438</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>-329292</v>
+        <v>-373957</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>-342791</v>
+        <v>-283493</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-360637</v>
+        <v>-333680</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-389971</v>
+        <v>-367402</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>-396407</v>
+        <v>-451158</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>-433860</v>
+        <v>-489571</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>-459526</v>
+        <v>-424143</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-303473</v>
+        <v>-281873</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>-271304</v>
+        <v>-309625</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>-302483</v>
+        <v>-341903</v>
       </c>
     </row>
     <row r="9">
@@ -3073,40 +3087,40 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-219542</v>
+        <v>-241084</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-235320</v>
+        <v>-193203</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-264975</v>
+        <v>-259882</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-276195</v>
+        <v>-275444</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>-292917</v>
+        <v>-322296</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>-319063</v>
+        <v>-255508</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>-324260</v>
+        <v>-317552</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>-352286</v>
+        <v>-345672</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>-370219</v>
+        <v>-408157</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-259642</v>
+        <v>-284448</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>-233632</v>
+        <v>-228541</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>-261290</v>
+        <v>-255963</v>
       </c>
     </row>
     <row r="10">
@@ -3177,40 +3191,40 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-332205</v>
+        <v>-344528</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-348157</v>
+        <v>-372816</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-398939</v>
+        <v>-364678</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-433206</v>
+        <v>-421264</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-471593</v>
+        <v>-489531</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-507686</v>
+        <v>-525634</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>-496244</v>
+        <v>-452484</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-522575</v>
+        <v>-479924</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-552532</v>
+        <v>-574095</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-358586</v>
+        <v>-371568</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>-330272</v>
+        <v>-362433</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>-363239</v>
+        <v>-332838</v>
       </c>
     </row>
     <row r="12">
@@ -3229,40 +3243,40 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-108721</v>
+        <v>-96647</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-113942</v>
+        <v>-105744</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-130562</v>
+        <v>-143219</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>-141776</v>
+        <v>-163265</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-154340</v>
+        <v>-136765</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>-166152</v>
+        <v>-148568</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>-162407</v>
+        <v>-178574</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>-171024</v>
+        <v>-186781</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>-180829</v>
+        <v>-159703</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-117356</v>
+        <v>-104637</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>-108088</v>
+        <v>-103142</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>-118878</v>
+        <v>-130109</v>
       </c>
     </row>
     <row r="13">
@@ -3281,40 +3295,40 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-65233</v>
+        <v>-69264</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-68365</v>
+        <v>-74834</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-78337</v>
+        <v>-73655</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>-85066</v>
+        <v>-84898</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>-92604</v>
+        <v>-98471</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>-99691</v>
+        <v>-105561</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>-97444</v>
+        <v>-91464</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>-102614</v>
+        <v>-96786</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-108497</v>
+        <v>-115549</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-70414</v>
+        <v>-74660</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>-64853</v>
+        <v>-52603</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>-71327</v>
+        <v>-67173</v>
       </c>
     </row>
     <row r="14">
@@ -3333,40 +3347,40 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-43489</v>
+        <v>-39733</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-45577</v>
+        <v>-43382</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-52225</v>
+        <v>-58652</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>-56711</v>
+        <v>-66758</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>-61736</v>
+        <v>-56269</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>-66460</v>
+        <v>-60990</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>-64963</v>
+        <v>-73172</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>-68410</v>
+        <v>-76411</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>-72332</v>
+        <v>-65760</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-46942</v>
+        <v>-42985</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>-43235</v>
+        <v>-42288</v>
       </c>
       <c r="P14" s="2" t="n">
-        <v>-47552</v>
+        <v>-53255</v>
       </c>
     </row>
     <row r="15">
@@ -3385,40 +3399,40 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-86977</v>
+        <v>-94499</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-91154</v>
+        <v>-73750</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>-104450</v>
+        <v>-100936</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>-113421</v>
+        <v>-116100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>-123472</v>
+        <v>-134421</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>-132921</v>
+        <v>-143875</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>-129925</v>
+        <v>-125436</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>-136820</v>
+        <v>-132445</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>-144663</v>
+        <v>-157824</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-93884</v>
+        <v>-101808</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>-86471</v>
+        <v>-72200</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>-95103</v>
+        <v>-91985</v>
       </c>
     </row>
     <row r="16">
@@ -3437,40 +3451,40 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>-130466</v>
+        <v>-122420</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-136731</v>
+        <v>-133400</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>-156675</v>
+        <v>-180048</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>-170133</v>
+        <v>-148028</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>-185208</v>
+        <v>-173496</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>-199382</v>
+        <v>-187664</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>-194889</v>
+        <v>-224742</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>-205230</v>
+        <v>-234326</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>-216995</v>
+        <v>-202917</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-140825</v>
+        <v>-132349</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>-129708</v>
+        <v>-129961</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>-142654</v>
+        <v>-163393</v>
       </c>
     </row>
     <row r="17">
@@ -3658,40 +3672,40 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5419084</v>
+        <v>5183580</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>5814226</v>
+        <v>5980898</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>6604509</v>
+        <v>6780275</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>6943201</v>
+        <v>7496975</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>7366568</v>
+        <v>7037935</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>7959280</v>
+        <v>7630390</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>8015729</v>
+        <v>8234269</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>8693115</v>
+        <v>8913922</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>9201154</v>
+        <v>8779487</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>9523194</v>
+        <v>9119763</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>5029587</v>
+        <v>5170152</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>5588430</v>
+        <v>5733688</v>
       </c>
     </row>
     <row r="3">
@@ -3710,40 +3724,40 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1912618</v>
+        <v>2175621</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2052080</v>
+        <v>1794270</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2331003</v>
+        <v>2059126</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>2450542</v>
+        <v>2300862</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>2599965</v>
+        <v>2966972</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2809158</v>
+        <v>3176452</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>2829081</v>
+        <v>2491040</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>3068158</v>
+        <v>2726611</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>3247466</v>
+        <v>3718371</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>3361127</v>
+        <v>3811666</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>1775149</v>
+        <v>1557722</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>1972387</v>
+        <v>1747701</v>
       </c>
     </row>
     <row r="4">
@@ -3762,40 +3776,40 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1561971</v>
+        <v>1534472</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1675866</v>
+        <v>1767004</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1903653</v>
+        <v>1999764</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2001276</v>
+        <v>1597182</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>2123305</v>
+        <v>2084931</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2294146</v>
+        <v>2255742</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>2310416</v>
+        <v>2429917</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>2505662</v>
+        <v>2626402</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>2652097</v>
+        <v>2602859</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>2744921</v>
+        <v>2697813</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>1449704</v>
+        <v>1526566</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1610783</v>
+        <v>1690211</v>
       </c>
     </row>
     <row r="5">
@@ -3814,40 +3828,40 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-3380117</v>
+        <v>-3547296</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-3669998</v>
+        <v>-3968147</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-4178479</v>
+        <v>-3878941</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>-4351874</v>
+        <v>-4125973</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-4559599</v>
+        <v>-4790005</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>-4906040</v>
+        <v>-5205535</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>-4981323</v>
+        <v>-4611191</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>-5472034</v>
+        <v>-5097029</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-5825133</v>
+        <v>-6125054</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-6007308</v>
+        <v>-6294676</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>-3105575</v>
+        <v>-2869134</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>-3448816</v>
+        <v>-3205248</v>
       </c>
     </row>
     <row r="6">
@@ -3866,40 +3880,40 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-2104735</v>
+        <v>-1900624</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-2259530</v>
+        <v>-2124429</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-2550985</v>
+        <v>-2828583</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>-2662430</v>
+        <v>-2977293</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>-2820033</v>
+        <v>-2539316</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>-3063606</v>
+        <v>-2817210</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>-3108639</v>
+        <v>-3453186</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>-3380439</v>
+        <v>-3728810</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>-3561655</v>
+        <v>-3196982</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-3676580</v>
+        <v>-3327119</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>-1927212</v>
+        <v>-2147056</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>-2155881</v>
+        <v>-2382688</v>
       </c>
     </row>
     <row r="7">
@@ -3918,40 +3932,40 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-446803</v>
+        <v>-479806</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-481929</v>
+        <v>-385147</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>-544684</v>
+        <v>-519683</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>-566450</v>
+        <v>-550817</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>-596986</v>
+        <v>-642085</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>-647416</v>
+        <v>-702204</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>-658970</v>
+        <v>-627435</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>-720201</v>
+        <v>-688499</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-760639</v>
+        <v>-819310</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-784451</v>
+        <v>-840658</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>-407578</v>
+        <v>-387622</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>-455792</v>
+        <v>-435051</v>
       </c>
     </row>
     <row r="8">
@@ -3970,40 +3984,40 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-326000</v>
+        <v>-302342</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-352475</v>
+        <v>-339685</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>-399616</v>
+        <v>-453407</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>-416008</v>
+        <v>-343848</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-437531</v>
+        <v>-404921</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-472947</v>
+        <v>-446061</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>-480714</v>
+        <v>-546708</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>-526280</v>
+        <v>-593416</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>-557619</v>
+        <v>-514826</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-575125</v>
+        <v>-534155</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>-298434</v>
+        <v>-340587</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>-332731</v>
+        <v>-376093</v>
       </c>
     </row>
     <row r="9">
@@ -4022,40 +4036,40 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-280724</v>
+        <v>-308311</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-301583</v>
+        <v>-248107</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-340597</v>
+        <v>-333747</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-355355</v>
+        <v>-354186</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>-376119</v>
+        <v>-413941</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>-408435</v>
+        <v>-327434</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>-414548</v>
+        <v>-405674</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>-451108</v>
+        <v>-442308</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>-475526</v>
+        <v>-524400</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-490818</v>
+        <v>-537674</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>-256996</v>
+        <v>-251396</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>-287419</v>
+        <v>-281559</v>
       </c>
     </row>
     <row r="10">
@@ -4126,40 +4140,40 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-374214</v>
+        <v>-388097</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-390418</v>
+        <v>-418070</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-446018</v>
+        <v>-407714</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-485003</v>
+        <v>-471634</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-530224</v>
+        <v>-550393</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-572684</v>
+        <v>-592929</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>-559502</v>
+        <v>-510164</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-586793</v>
+        <v>-538900</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-618018</v>
+        <v>-642136</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-647922</v>
+        <v>-671379</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>-363299</v>
+        <v>-398676</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>-399563</v>
+        <v>-366123</v>
       </c>
     </row>
     <row r="12">
@@ -4178,40 +4192,40 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-122470</v>
+        <v>-108869</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-127773</v>
+        <v>-118580</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-145970</v>
+        <v>-160121</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>-158728</v>
+        <v>-182786</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-173528</v>
+        <v>-153768</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>-187424</v>
+        <v>-167588</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>-183110</v>
+        <v>-201338</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>-192041</v>
+        <v>-209734</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>-202261</v>
+        <v>-178631</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-212047</v>
+        <v>-189065</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>-118898</v>
+        <v>-113457</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>-130765</v>
+        <v>-143119</v>
       </c>
     </row>
     <row r="13">
@@ -4230,40 +4244,40 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-73482</v>
+        <v>-78022</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-76664</v>
+        <v>-83918</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-87582</v>
+        <v>-82348</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>-95237</v>
+        <v>-95049</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>-104117</v>
+        <v>-110713</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>-112454</v>
+        <v>-119076</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>-109866</v>
+        <v>-103124</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>-115225</v>
+        <v>-108681</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-121356</v>
+        <v>-129244</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-127229</v>
+        <v>-134901</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>-71338</v>
+        <v>-57863</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>-78461</v>
+        <v>-73891</v>
       </c>
     </row>
     <row r="14">
@@ -4282,40 +4296,40 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-48988</v>
+        <v>-44757</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-51109</v>
+        <v>-48648</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-58388</v>
+        <v>-65573</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>-63492</v>
+        <v>-74740</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>-69411</v>
+        <v>-63264</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>-74970</v>
+        <v>-68800</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>-73243</v>
+        <v>-82498</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>-76816</v>
+        <v>-85800</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>-80904</v>
+        <v>-73554</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-84819</v>
+        <v>-77670</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>-47559</v>
+        <v>-46517</v>
       </c>
       <c r="P14" s="2" t="n">
-        <v>-52307</v>
+        <v>-58580</v>
       </c>
     </row>
     <row r="15">
@@ -4334,40 +4348,40 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-97976</v>
+        <v>-106449</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-102219</v>
+        <v>-82702</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>-116776</v>
+        <v>-112847</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>-126982</v>
+        <v>-129981</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>-138822</v>
+        <v>-151132</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>-149939</v>
+        <v>-162296</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>-146488</v>
+        <v>-141427</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>-153633</v>
+        <v>-148721</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>-161808</v>
+        <v>-176529</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-169638</v>
+        <v>-183955</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>-95117</v>
+        <v>-79419</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>-104613</v>
+        <v>-101183</v>
       </c>
     </row>
     <row r="16">
@@ -4386,40 +4400,40 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>-146966</v>
+        <v>-137902</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-153328</v>
+        <v>-149593</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>-175163</v>
+        <v>-201294</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>-190474</v>
+        <v>-165726</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>-208233</v>
+        <v>-195065</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>-224909</v>
+        <v>-211691</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>-219731</v>
+        <v>-253389</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>-230450</v>
+        <v>-263122</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>-242712</v>
+        <v>-226965</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-254456</v>
+        <v>-239141</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>-142679</v>
+        <v>-142958</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>-156919</v>
+        <v>-179732</v>
       </c>
     </row>
     <row r="17">
@@ -4607,40 +4621,40 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4985557</v>
+        <v>4768894</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>5349088</v>
+        <v>5502427</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>6076148</v>
+        <v>6237853</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>6387745</v>
+        <v>6897217</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>6777243</v>
+        <v>6474900</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>7322538</v>
+        <v>7019959</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>7374471</v>
+        <v>7575528</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>7997666</v>
+        <v>8200808</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>8465062</v>
+        <v>8077129</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>8761338</v>
+        <v>8390182</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>4627220</v>
+        <v>4756540</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>5141356</v>
+        <v>5274993</v>
       </c>
     </row>
     <row r="3">
@@ -4659,40 +4673,40 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1759609</v>
+        <v>2001572</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1887914</v>
+        <v>1650728</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2144523</v>
+        <v>1894396</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>2254499</v>
+        <v>2116794</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>2391968</v>
+        <v>2729615</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2584425</v>
+        <v>2922336</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>2602755</v>
+        <v>2291757</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>2822705</v>
+        <v>2508482</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>2987669</v>
+        <v>3420901</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>3092237</v>
+        <v>3506733</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>1633137</v>
+        <v>1433104</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>1814596</v>
+        <v>1607885</v>
       </c>
     </row>
     <row r="4">
@@ -4711,40 +4725,40 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1437013</v>
+        <v>1411713</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1541797</v>
+        <v>1625644</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1751361</v>
+        <v>1839783</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1841174</v>
+        <v>1469407</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1953441</v>
+        <v>1918137</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2110614</v>
+        <v>2075282</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>2125583</v>
+        <v>2235524</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>2305209</v>
+        <v>2416290</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>2439929</v>
+        <v>2394630</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>2525327</v>
+        <v>2481987</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>1333728</v>
+        <v>1404441</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1481920</v>
+        <v>1554994</v>
       </c>
     </row>
     <row r="5">
@@ -4763,40 +4777,40 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-3211111</v>
+        <v>-3369930</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-3486498</v>
+        <v>-3769740</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-3969555</v>
+        <v>-3684995</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>-4134280</v>
+        <v>-3919674</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-4331619</v>
+        <v>-4550505</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>-4660738</v>
+        <v>-4945259</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>-4732257</v>
+        <v>-4380633</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>-5198432</v>
+        <v>-4842177</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-5533876</v>
+        <v>-5818802</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-5706943</v>
+        <v>-5979943</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>-2950296</v>
+        <v>-2725678</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>-3276375</v>
+        <v>-3044985</v>
       </c>
     </row>
     <row r="6">
@@ -4815,40 +4829,40 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-1999498</v>
+        <v>-1805593</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-2146554</v>
+        <v>-2018208</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-2423436</v>
+        <v>-2687154</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>-2529309</v>
+        <v>-2828429</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>-2679031</v>
+        <v>-2412350</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>-2910426</v>
+        <v>-2676350</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>-2953207</v>
+        <v>-3280527</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>-3211417</v>
+        <v>-3542370</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>-3383572</v>
+        <v>-3037132</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-3492751</v>
+        <v>-3160763</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>-1830851</v>
+        <v>-2039702</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>-2048087</v>
+        <v>-2263554</v>
       </c>
     </row>
     <row r="7">
@@ -4867,40 +4881,40 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-424463</v>
+        <v>-455816</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-457833</v>
+        <v>-365890</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>-517450</v>
+        <v>-493699</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>-538128</v>
+        <v>-523276</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>-567137</v>
+        <v>-609981</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>-615045</v>
+        <v>-667093</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>-626022</v>
+        <v>-596063</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>-684191</v>
+        <v>-654074</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-722607</v>
+        <v>-778344</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-745228</v>
+        <v>-798624</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>-387199</v>
+        <v>-368241</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>-433002</v>
+        <v>-413298</v>
       </c>
     </row>
     <row r="8">
@@ -4919,40 +4933,40 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-309700</v>
+        <v>-287225</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-334851</v>
+        <v>-322700</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>-379635</v>
+        <v>-430736</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>-395208</v>
+        <v>-326656</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-415654</v>
+        <v>-384675</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-449300</v>
+        <v>-423758</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>-456678</v>
+        <v>-519372</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>-499966</v>
+        <v>-563745</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>-529738</v>
+        <v>-489084</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-546369</v>
+        <v>-507448</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>-283512</v>
+        <v>-323557</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>-316094</v>
+        <v>-357288</v>
       </c>
     </row>
     <row r="9">
@@ -4971,40 +4985,40 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-266688</v>
+        <v>-292896</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-286504</v>
+        <v>-235702</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-323567</v>
+        <v>-317059</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-337587</v>
+        <v>-336477</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>-357313</v>
+        <v>-393243</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>-388013</v>
+        <v>-311062</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>-393821</v>
+        <v>-385390</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>-428553</v>
+        <v>-420193</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>-451750</v>
+        <v>-498181</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-466277</v>
+        <v>-510790</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>-244146</v>
+        <v>-238826</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>-273048</v>
+        <v>-267481</v>
       </c>
     </row>
     <row r="10">
@@ -5075,40 +5089,40 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-381698</v>
+        <v>-395858</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-398226</v>
+        <v>-426431</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-454938</v>
+        <v>-415868</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-494703</v>
+        <v>-481067</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-540828</v>
+        <v>-561399</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-584138</v>
+        <v>-604789</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>-570692</v>
+        <v>-520367</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-598529</v>
+        <v>-549680</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-630378</v>
+        <v>-654979</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-660880</v>
+        <v>-684805</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>-370565</v>
+        <v>-406650</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>-407554</v>
+        <v>-373444</v>
       </c>
     </row>
     <row r="12">
@@ -5127,40 +5141,40 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-124919</v>
+        <v>-111046</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-130328</v>
+        <v>-120951</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-148889</v>
+        <v>-163323</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>-161903</v>
+        <v>-186442</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-176999</v>
+        <v>-156844</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>-191172</v>
+        <v>-170940</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>-186772</v>
+        <v>-205364</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>-195882</v>
+        <v>-213929</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>-206306</v>
+        <v>-182203</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-216288</v>
+        <v>-192846</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>-121276</v>
+        <v>-115727</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>-133380</v>
+        <v>-145981</v>
       </c>
     </row>
     <row r="13">
@@ -5179,40 +5193,40 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-74952</v>
+        <v>-79583</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-78197</v>
+        <v>-85596</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-89334</v>
+        <v>-83995</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>-97142</v>
+        <v>-96950</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>-106199</v>
+        <v>-112927</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>-114703</v>
+        <v>-121457</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>-112063</v>
+        <v>-105186</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>-117530</v>
+        <v>-110855</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-123783</v>
+        <v>-131829</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-129774</v>
+        <v>-137600</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>-72765</v>
+        <v>-59020</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>-80030</v>
+        <v>-75369</v>
       </c>
     </row>
     <row r="14">
@@ -5231,40 +5245,40 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-49968</v>
+        <v>-45652</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-52131</v>
+        <v>-49621</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-59556</v>
+        <v>-66885</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>-64762</v>
+        <v>-76235</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>-70799</v>
+        <v>-64530</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>-76469</v>
+        <v>-70175</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>-74708</v>
+        <v>-84148</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>-78352</v>
+        <v>-87515</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>-82522</v>
+        <v>-75025</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-86515</v>
+        <v>-79223</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>-48510</v>
+        <v>-47447</v>
       </c>
       <c r="P14" s="2" t="n">
-        <v>-53353</v>
+        <v>-59752</v>
       </c>
     </row>
     <row r="15">
@@ -5283,40 +5297,40 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-99936</v>
+        <v>-108579</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-104263</v>
+        <v>-84356</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>-119112</v>
+        <v>-115105</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>-129522</v>
+        <v>-132581</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>-141598</v>
+        <v>-154154</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>-152938</v>
+        <v>-165542</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>-149418</v>
+        <v>-144256</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>-156706</v>
+        <v>-151695</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>-165044</v>
+        <v>-180059</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-173031</v>
+        <v>-187635</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>-97019</v>
+        <v>-81007</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>-106705</v>
+        <v>-103206</v>
       </c>
     </row>
     <row r="16">
@@ -5335,40 +5349,40 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>-149905</v>
+        <v>-140660</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-156395</v>
+        <v>-152585</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>-178666</v>
+        <v>-205319</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>-194283</v>
+        <v>-169040</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>-212398</v>
+        <v>-198967</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>-229407</v>
+        <v>-215924</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>-224126</v>
+        <v>-258458</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>-235059</v>
+        <v>-268384</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>-247566</v>
+        <v>-231504</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-259545</v>
+        <v>-243924</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>-145533</v>
+        <v>-145817</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>-160057</v>
+        <v>-183327</v>
       </c>
     </row>
     <row r="17">
@@ -5556,40 +5570,40 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5960992</v>
+        <v>5701938</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>6395649</v>
+        <v>6578988</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>7264960</v>
+        <v>7458303</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>7637521</v>
+        <v>8246673</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>8103225</v>
+        <v>7741729</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>8755208</v>
+        <v>8393429</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>8817302</v>
+        <v>9057696</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>9562427</v>
+        <v>9805315</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>10121269</v>
+        <v>9657435</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10475513</v>
+        <v>10031740</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>5532546</v>
+        <v>5687167</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>6147273</v>
+        <v>6307056</v>
       </c>
     </row>
     <row r="3">
@@ -5608,40 +5622,40 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2103880</v>
+        <v>2393183</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2257288</v>
+        <v>1973697</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2564103</v>
+        <v>2265038</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>2695596</v>
+        <v>2530948</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>2859962</v>
+        <v>3263670</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>3090074</v>
+        <v>3494098</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>3111989</v>
+        <v>2740144</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>3374974</v>
+        <v>2999272</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>3572213</v>
+        <v>4090208</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>3697240</v>
+        <v>4192832</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>1952664</v>
+        <v>1713494</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>2169626</v>
+        <v>1922472</v>
       </c>
     </row>
     <row r="4">
@@ -5660,40 +5674,40 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1718168</v>
+        <v>1687919</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1843453</v>
+        <v>1943705</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>2094018</v>
+        <v>2199740</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2201404</v>
+        <v>1756900</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>2335636</v>
+        <v>2293424</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2523561</v>
+        <v>2481316</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>2541458</v>
+        <v>2672909</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>2756228</v>
+        <v>2889042</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>2917307</v>
+        <v>2863146</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>3019413</v>
+        <v>2967594</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>1594674</v>
+        <v>1679223</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1771861</v>
+        <v>1859232</v>
       </c>
     </row>
     <row r="5">
@@ -5712,40 +5726,40 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-3582924</v>
+        <v>-3760134</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-3890198</v>
+        <v>-4206236</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-4429188</v>
+        <v>-4111679</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>-4612986</v>
+        <v>-4373531</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-4833175</v>
+        <v>-5077405</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>-5200402</v>
+        <v>-5517866</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>-5280202</v>
+        <v>-4887862</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>-5800356</v>
+        <v>-5402851</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-6174641</v>
+        <v>-6492558</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-6367746</v>
+        <v>-6672356</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>-3291910</v>
+        <v>-3041283</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>-3655745</v>
+        <v>-3397562</v>
       </c>
     </row>
     <row r="6">
@@ -5764,40 +5778,40 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-2231019</v>
+        <v>-2014662</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-2395102</v>
+        <v>-2251895</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-2704044</v>
+        <v>-2998297</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>-2822176</v>
+        <v>-3155931</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>-2989235</v>
+        <v>-2691675</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>-3247422</v>
+        <v>-2986243</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>-3295157</v>
+        <v>-3660377</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>-3583265</v>
+        <v>-3952539</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>-3775354</v>
+        <v>-3388800</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-3897175</v>
+        <v>-3526747</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>-2042845</v>
+        <v>-2275879</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>-2285234</v>
+        <v>-2525650</v>
       </c>
     </row>
     <row r="7">
@@ -5816,40 +5830,40 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-473611</v>
+        <v>-508594</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-510845</v>
+        <v>-408256</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>-577365</v>
+        <v>-550864</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>-600437</v>
+        <v>-583866</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>-632805</v>
+        <v>-680610</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>-686261</v>
+        <v>-744336</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>-698508</v>
+        <v>-665081</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>-763413</v>
+        <v>-729808</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-806277</v>
+        <v>-868468</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-831518</v>
+        <v>-891097</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>-432033</v>
+        <v>-410880</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>-483140</v>
+        <v>-461154</v>
       </c>
     </row>
     <row r="8">
@@ -5868,40 +5882,40 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-345560</v>
+        <v>-320482</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-373624</v>
+        <v>-360067</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>-423593</v>
+        <v>-480611</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>-440968</v>
+        <v>-364478</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-463783</v>
+        <v>-429217</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-501324</v>
+        <v>-472825</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>-509557</v>
+        <v>-579511</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>-557857</v>
+        <v>-629021</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>-591076</v>
+        <v>-545715</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-609633</v>
+        <v>-566205</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>-316340</v>
+        <v>-361022</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>-352695</v>
+        <v>-398659</v>
       </c>
     </row>
     <row r="9">
@@ -5920,40 +5934,40 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-297567</v>
+        <v>-326809</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-319678</v>
+        <v>-262993</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-361033</v>
+        <v>-353772</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-376676</v>
+        <v>-375437</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>-398686</v>
+        <v>-438777</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>-432941</v>
+        <v>-347080</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>-439421</v>
+        <v>-430014</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>-478174</v>
+        <v>-468846</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>-504058</v>
+        <v>-555865</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-520267</v>
+        <v>-569934</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>-272416</v>
+        <v>-266480</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>-304664</v>
+        <v>-298453</v>
       </c>
     </row>
     <row r="10">
@@ -6024,40 +6038,40 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-385440</v>
+        <v>-399739</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-402131</v>
+        <v>-430612</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-459399</v>
+        <v>-419946</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-499553</v>
+        <v>-485782</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-546131</v>
+        <v>-566905</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-589865</v>
+        <v>-610718</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>-576287</v>
+        <v>-525468</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-604397</v>
+        <v>-555069</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-636559</v>
+        <v>-661401</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-667360</v>
+        <v>-691522</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>-374198</v>
+        <v>-410637</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>-411550</v>
+        <v>-377106</v>
       </c>
     </row>
     <row r="12">
@@ -6076,40 +6090,40 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-126144</v>
+        <v>-112135</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-131606</v>
+        <v>-122137</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-150349</v>
+        <v>-164924</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>-163490</v>
+        <v>-188270</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-178734</v>
+        <v>-158381</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>-193047</v>
+        <v>-172616</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>-188603</v>
+        <v>-207377</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>-197802</v>
+        <v>-216026</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>-208329</v>
+        <v>-183990</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-218408</v>
+        <v>-194736</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>-122465</v>
+        <v>-116861</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>-134688</v>
+        <v>-147413</v>
       </c>
     </row>
     <row r="13">
@@ -6128,40 +6142,40 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-75686</v>
+        <v>-80363</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-78964</v>
+        <v>-86436</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-90209</v>
+        <v>-84818</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>-98094</v>
+        <v>-97900</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>-107241</v>
+        <v>-114035</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>-115828</v>
+        <v>-122648</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>-113162</v>
+        <v>-106218</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>-118682</v>
+        <v>-111941</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-124997</v>
+        <v>-133122</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-131046</v>
+        <v>-138948</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>-73478</v>
+        <v>-59598</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>-80815</v>
+        <v>-76108</v>
       </c>
     </row>
     <row r="14">
@@ -6180,40 +6194,40 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-50458</v>
+        <v>-46100</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-52642</v>
+        <v>-50107</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-60140</v>
+        <v>-67541</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>-65397</v>
+        <v>-76983</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>-71493</v>
+        <v>-65162</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>-77219</v>
+        <v>-70864</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>-75440</v>
+        <v>-84973</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>-79120</v>
+        <v>-88373</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>-83331</v>
+        <v>-75760</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-87364</v>
+        <v>-80000</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>-48986</v>
+        <v>-47913</v>
       </c>
       <c r="P14" s="2" t="n">
-        <v>-53876</v>
+        <v>-60337</v>
       </c>
     </row>
     <row r="15">
@@ -6232,40 +6246,40 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-100915</v>
+        <v>-109642</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-105286</v>
+        <v>-85184</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>-120279</v>
+        <v>-116232</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>-130791</v>
+        <v>-133880</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>-142987</v>
+        <v>-155666</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>-154437</v>
+        <v>-167165</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>-150883</v>
+        <v>-145671</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>-158242</v>
+        <v>-153182</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>-166662</v>
+        <v>-181824</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-174727</v>
+        <v>-189474</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>-97971</v>
+        <v>-81802</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>-107751</v>
+        <v>-104218</v>
       </c>
     </row>
     <row r="16">
@@ -6284,40 +6298,40 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>-151375</v>
+        <v>-142039</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-157928</v>
+        <v>-154081</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>-180418</v>
+        <v>-207333</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>-196188</v>
+        <v>-170698</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>-214480</v>
+        <v>-200917</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>-231656</v>
+        <v>-218041</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>-226323</v>
+        <v>-260991</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>-237364</v>
+        <v>-271016</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>-249993</v>
+        <v>-233774</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-262090</v>
+        <v>-246315</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>-146959</v>
+        <v>-147246</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>-161627</v>
+        <v>-185125</v>
       </c>
     </row>
     <row r="17">

</xml_diff>